<commit_message>
Track 2: mechanism characterisation and drug repurposing hypotheses
Mechanism: BubR1 is a vertebrate pseudokinase; both alleles reduce functional
dosage of a scaffolding module. Open Targets finds no druggable pocket, which
is why no docking was performed.

Candidates: dasatinib (senolytic, FDA-approved with pediatric + concomitant-
chemotherapy labelling), sirolimus/everolimus (mTORC1), readthrough (ranked
third). Argues against SAC-directed synthetic lethality in constitutional
checkpoint deficiency.

Adds ptc_triage.py, a generalisable readthrough-amenability triage, plus the
3-minute pitch script and slides. No patient sequence data.
</commit_message>
<xml_diff>
--- a/submission/checkpoint-in-trans_methods_description.xlsx
+++ b/submission/checkpoint-in-trans_methods_description.xlsx
@@ -726,7 +726,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="64" customWidth="1" style="7" min="1" max="1"/>
-    <col width="45" customWidth="1" style="7" min="2" max="2"/>
+    <col width="100" customWidth="1" style="7" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1" s="7">
@@ -759,7 +759,11 @@
           <t>Team name</t>
         </is>
       </c>
-      <c r="B7" s="3" t="n"/>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>checkpoint-in-trans</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="30" customHeight="1" s="7">
       <c r="A8" s="2" t="inlineStr">
@@ -767,7 +771,15 @@
           <t>Please describe your approach in detail (how you went from variant/mechanism to candidate medication(s)).</t>
         </is>
       </c>
-      <c r="B8" s="3" t="n"/>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>From lesion to candidate in four steps.
+1) Establish what is broken. Structured extraction over PubMed abstracts to settle whether the BubR1 C-terminal domain is catalytically active; structural placement of both variants on the AlphaFold model of O60566 and on the two cryo-EM APC/C-MCC structures that align to the region; codon-level characterisation of the premature stop from the RefSeq CDS; mapping of UniProt functional elements onto the truncation point.
+2) Establish that the protein itself is not a target. Open Targets tractability across 28 buckets, read together with the pseudokinase finding and the 34.7 A distance from the nucleotide site. This is what ruled docking out: no pocket, and the required direction is restoration rather than inhibition.
+3) Generate candidates from mechanism, not from similarity. Four PubMed axes - BubR1 and senescence/progeria, senolytic intervention, stop-codon readthrough, and spindle-poison response in checkpoint-deficient cells - each with structured extraction into a table, then regulatory status from openFDA.
+4) Test each candidate against the specific lesion rather than the gene. For readthrough this meant asking what residue the drug would actually install and whether 247 vertebrate orthologs tolerate it at that position; the answer reordered the ranking.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="60" customHeight="1" s="7">
       <c r="A9" s="5" t="inlineStr">
@@ -775,7 +787,11 @@
           <t>(required) If commercially-available Generative AI was used, record the provider, the plan or tier, and the relevant setting in your methods description. A line is enough, for example, "Anthropic API, Claude Sonnet, commercial terms, no training on customer content."</t>
         </is>
       </c>
-      <c r="B9" s="3" t="n"/>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Anthropic, Claude Opus 5, accessed through a Team/Enterprise plan on the Claude Science platform, under commercial terms with no training on customer content.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="45" customHeight="1" s="7">
       <c r="A10" s="4" t="inlineStr">
@@ -783,7 +799,11 @@
           <t>Was candidate identification automated (e.g., via a drug-target database query or LLM-assisted search), or primarily manual literature review and expert curation?</t>
         </is>
       </c>
-      <c r="B10" s="3" t="n"/>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Both, and the split is worth stating precisely. Retrieval and extraction were AUTOMATED: PubMed E-utilities queries, LLM-assisted structured extraction of each abstract into typed fields, openFDA and Open Targets queries, structural computation, and the 247-ortholog alignment. Candidate selection, ranking, and the decision to argue against one strategy were EXPERT CURATION on top of those outputs.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -791,7 +811,14 @@
           <t>Please describe any manual literature review or expert curation in detail.</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n"/>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Three components are expert judgement rather than pipeline output.
+(a) Ranking. Candidates are ordered by the strength of the mechanistic chain from this proband's specific lesion, not by database score. Readthrough was placed third despite being the only axis addressing the causal lesion, because the ortholog analysis showed the product is non-conservative and the regulatory check showed no approved medicine remains.
+(b) Contradiction handling. Where sources disagree we report the split rather than resolve it: spindle-poison response in checkpoint-weakened cells (30 abstracts 'more sensitive' vs 18 'more resistant'), and the BubR1-mTOR direction (progeroid mice vs hepatocellular carcinoma).
+(c) The contraindication. No database returns 'do not do this'. That SAC-directed synthetic lethality is hazardous in a constitutional checkpoint deficiency is an inference from the structure of the therapeutic window, and we include it because a clinical team needs it.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="45" customHeight="1" s="7">
       <c r="A12" s="4" t="inlineStr">
@@ -799,7 +826,11 @@
           <t>Please state whether you relied solely on publicly available drug/target databases and literature (preferred), or whether proprietary data sources were also used.</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Publicly available drug, target and literature sources only. No proprietary data were used.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="30" customHeight="1" s="7">
       <c r="A13" s="4" t="inlineStr">
@@ -807,7 +838,11 @@
           <t>Please describe the public data sources used in detail (e.g., DrugBank, ChEMBL, ClinicalTrials.gov, OMIM, PubMed literature search).</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n"/>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>PubMed via NCBI E-utilities (five query axes; 98 readthrough, 158 senescence/senolytic, 55 mTOR/MVA-treatment, 77 spindle-poison and 35 kinase-activity abstracts retrieved and extracted into structured tables, all shipped in the repository). openFDA Drugs@FDA and SPL labels for approval status, marketing status and pediatric indications. Open Targets GraphQL for target tractability. UniProt (O60566) for domain and feature annotation and for the 247 vertebrate BUB1B orthologs used in the conservation analysis. AlphaFold DB (AF-O60566, v6) for structure. RCSB PDB for the experimental structures (6TLJ, 5KHU and seven other BUB1B entities). RefSeq NM_001211.6 for the CDS. EMA and European Commission public records for the Translarna authorisation status. Software: Biopython (PairwiseAligner with BLOSUM62, Shrake-Rupley SASA), NumPy, pandas, matplotlib.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -815,7 +850,11 @@
           <t>Please describe any proprietary data sources used in detail.</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="30" customHeight="1" s="7">
       <c r="A15" s="4" t="inlineStr">
@@ -823,7 +862,15 @@
           <t>How did you characterize the variant's mechanism (e.g., loss-of-function vs. gain-of-function, pathway disrupted, downstream biological consequence)?</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Loss of function, by dosage insufficiency, of a scaffolding module - established on four independent lines rather than asserted.
+Direction: both alleles reduce functional protein. p.Leu737Ter removes the entire pseudokinase domain (766-1050) while retaining everything N-terminal, and sits 314 codons upstream of the natural stop, so the transcript is NMD-competent. p.Asn1002Lys buries a positive charge in an aromatic packing environment within the same domain.
+Pathway disrupted: the mitotic checkpoint complex and kinetochore signalling. The domain is catalytically dead in vertebrates but required to promote KARD phosphorylation and to maintain kinase-phosphatase balance at the outer kinetochore, so the defect is scaffolding, not enzymatic. This distinction is load-bearing: it is why an ATP-competitive approach would have been wrong.
+Downstream consequence: weakened spindle assembly checkpoint, chromosome missegregation, mosaic variegated aneuploidy, and - per the mouse models - cellular senescence accumulation with progeroid pathology plus embryonal-tumour predisposition. The senescence limb is what makes the lead candidate druggable, since BubR1 itself is not.
+Supporting evidence: Asn1002 is conserved in 226 of 247 vertebrate orthologs with lysine in none; the closest animal model, BubR1H/L1002P, reproduces the disease from the same allelic architecture.</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="30" customHeight="1" s="7">
       <c r="A16" s="4" t="inlineStr">
@@ -831,7 +878,11 @@
           <t>Please provide an estimate of time or effort spent on this analysis (if possible).</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n"/>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>This track: roughly 25 analysis cells in one working session, dominated by literature retrieval and extraction (423 abstracts across five axes) and by the 247-sequence pairwise alignment, which takes about nine seconds. All computation ran on 8 CPU cores with ~3 GiB RAM and no GPU; nothing here required one. The full project including Track 1 spans 56 hours of wall-clock time across 253 executed cells. LLM token cost is not visible from inside the analysis environment.</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="30" customHeight="1" s="7">
       <c r="A17" s="4" t="inlineStr">
@@ -839,7 +890,17 @@
           <t>Provide a method abstract (up to 500 words). Please include strengths and limitations of your approach as well as methodological detail.</t>
         </is>
       </c>
-      <c r="B17" s="3" t="n"/>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>The proband carries compound heterozygous BUB1B: p.Leu737Ter and p.Asn1002Lys, the pair submitted and confirmed in Track 1. We treated the case as dosage insufficiency of a scaffolding protein rather than a druggable lesion, which determined every subsequent choice.
+Mechanism. Structured extraction over PubMed abstracts established that vertebrate BubR1 is a pseudokinase: 13 of 16 abstracts taking a position report catalytic inactivity, the three dissenting ones being Drosophila where the enzyme is genuinely active. The C-terminal domain is nonetheless essential as a scaffold. On the AlphaFold model (local pLDDT 91.1) Asn1002 is 20% accessible, packs against Trp973/Phe977/Trp978/Phe997, and lies 34.7 A from the nucleotide site; neither cryo-EM structure of the APC/C-MCC complex resolves any of the 285 pseudokinase-domain residues. p.Leu737Ter removes the whole domain and is NMD-competent. Open Targets scores 28 tractability buckets with no pocket of high or medium quality.
+Candidates. (1) Senolytics, principally dasatinib. BubR1 insufficiency is the founding progeroid model of the senolytics field, and in BubR1H/L1002P mice - a reduced-protein allele plus a C-lobe pseudokinase missense, the same allelic architecture as this proband - progeroid severity tracked with SASP complexity. Dasatinib is FDA-approved with a pediatric indication from age 1, one of them in combination with chemotherapy. (2) mTORC1 inhibition, from the mTORC1 hyperactivity reported in the same mouse work. (3) Translational readthrough, ranked third.
+Innovation. Readthrough does not restore the wild-type residue; at UGA it inserts Trp, Cys or Arg. We therefore asked whether the protein tolerates the product. The PTC is TGA-A, the most permissive stop class, but across 247 vertebrate orthologs Leu occupies position 737 in 236 and none of the three insertable residues occurs in any species, at a position 90% buried. This demoted our own leading candidate. The step is packaged as ptc_triage.py and generalises to any nonsense allele.
+We also argue explicitly against SAC-directed synthetic lethality: its window depends on normal cells retaining an intact checkpoint, which is untrue in constitutional BUB1B insufficiency.
+Strengths. Every claim is traced to a retrieved source; the mechanism is grounded in structure and orthology rather than annotation (UniProt still lists EC 2.7.11.1, which the literature does not support); the negative and contraindication findings are reported as prominently as the positive ones; and the ranking was changed by our own analysis rather than defended.
+Limitations. No candidate has evidence in MVA, in this gene, or in children for this indication. The senolytic case rests on mouse genetics; the mTORC1 case is correlative and directionally inconsistent across contexts. No experimental structure covers either variant. Ortholog constraint is evolutionary evidence, not a functional assay. Near-cognate insertion frequencies were taken from the general literature, not measured for this context. Senescence is tumour-suppressive, and clearing it in a cancer-predisposition syndrome is the largest unresolved risk.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>